<commit_message>
feat(EM): add DeepSeek provider template
</commit_message>
<xml_diff>
--- a/Emmersive/package/LangMod/EN/emmersive_localizations.xlsx
+++ b/Emmersive/package/LangMod/EN/emmersive_localizations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\Elin.Plugins\Emmersive\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E64CF152-1A1A-415D-AFF9-263A9E2F95A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84A9C2FE-1A82-4CC9-9A1D-40BA3E8CC610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15960" yWindow="2685" windowWidth="26100" windowHeight="17625" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="28380" windowHeight="17610" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="340">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1053,6 +1053,28 @@
   </si>
   <si>
     <t>Player2を追加</t>
+  </si>
+  <si>
+    <t>Use Pieixan API</t>
+  </si>
+  <si>
+    <t>em_ui_add_service_piexian</t>
+  </si>
+  <si>
+    <t>em_ui_px_desc</t>
+  </si>
+  <si>
+    <t>贴吧群氕氙免费提供的站点
+模组群&lt;color=orange&gt;872068953&lt;/color&gt;</t>
+  </si>
+  <si>
+    <t>em_ui_add_service_deepseek</t>
+  </si>
+  <si>
+    <t>DeepSeek互換を追加</t>
+  </si>
+  <si>
+    <t>Add DeeSeek</t>
   </si>
 </sst>
 </file>
@@ -1418,7 +1440,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:XFC126"/>
+  <dimension ref="A1:XFC129"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="23.25"/>
   <cols>
     <col min="1" max="1" width="63.28515625" style="4" customWidth="1"/>
@@ -1562,847 +1584,847 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="4" t="s">
-        <v>20</v>
+        <v>337</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>142</v>
+        <v>338</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>141</v>
+        <v>339</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C15" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D15" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="15" spans="1:4" s="3" customFormat="1">
-      <c r="A15" s="4" t="s">
+    <row r="16" spans="1:4" s="3" customFormat="1">
+      <c r="A16" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4" t="s">
+      <c r="B16" s="4"/>
+      <c r="C16" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D16" s="4" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C18" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D18" s="4" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="46.5">
-      <c r="A18" s="4" t="s">
+    <row r="19" spans="1:4" ht="46.5">
+      <c r="A19" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C19" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D19" s="4" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="A19" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="4" t="s">
-        <v>96</v>
+        <v>30</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>97</v>
+        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="4" t="s">
-        <v>222</v>
+        <v>96</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>223</v>
+        <v>109</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>224</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="4" t="s">
-        <v>143</v>
+        <v>222</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>157</v>
+        <v>223</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>153</v>
+        <v>224</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>187</v>
+        <v>167</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>189</v>
+        <v>154</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
+      <c r="A33" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="C33" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="D32" s="4" t="s">
+      <c r="D33" s="4" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="69.75">
-      <c r="A33" s="4" t="s">
+    <row r="34" spans="1:4" ht="69.75">
+      <c r="A34" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C34" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D34" s="4" t="s">
         <v>173</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
-      <c r="A34" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C34" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="D34" s="4" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
+      <c r="A39" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C38" s="4" t="s">
+      <c r="C39" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="D38" s="4" t="s">
+      <c r="D39" s="4" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="39" spans="1:4" s="3" customFormat="1">
-      <c r="A39" s="4" t="s">
+    <row r="40" spans="1:4" s="3" customFormat="1">
+      <c r="A40" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B39" s="4"/>
-      <c r="C39" s="4" t="s">
+      <c r="B40" s="4"/>
+      <c r="C40" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D39" s="4" t="s">
+      <c r="D40" s="4" t="s">
         <v>76</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4">
-      <c r="A40" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="D40" s="4" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>116</v>
+        <v>136</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>77</v>
+        <v>137</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4">
+      <c r="A61" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C60" s="4" t="s">
+      <c r="C61" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="D60" s="4" t="s">
+      <c r="D61" s="4" t="s">
         <v>83</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" s="2" customFormat="1">
-      <c r="A61" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B61" s="4"/>
-      <c r="C61" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="D61" s="4" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="62" spans="1:4" s="2" customFormat="1">
       <c r="A62" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B62" s="4"/>
       <c r="C62" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" s="2" customFormat="1">
+      <c r="A63" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B63" s="4"/>
+      <c r="C63" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="D62" s="4" t="s">
+      <c r="D63" s="4" t="s">
         <v>85</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4">
-      <c r="A63" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C63" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="D63" s="4" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="64" spans="1:4">
       <c r="A64" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C64" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="4" t="s">
-        <v>175</v>
+        <v>70</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>176</v>
+        <v>134</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>176</v>
+        <v>95</v>
       </c>
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4">
+      <c r="A76" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C75" s="4" t="s">
+      <c r="C76" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="D75" s="4" t="s">
+      <c r="D76" s="4" t="s">
         <v>184</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" ht="46.5">
-      <c r="A76" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="C76" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="D76" s="4" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="77" spans="1:4" ht="46.5">
       <c r="A77" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" ht="46.5">
+      <c r="A78" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="C77" s="4" t="s">
+      <c r="C78" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="D77" s="4" t="s">
+      <c r="D78" s="4" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="78" spans="1:4">
-      <c r="A78" s="4" t="s">
+    <row r="79" spans="1:4">
+      <c r="A79" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="C78" s="4" t="s">
+      <c r="C79" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="D78" s="4" t="s">
+      <c r="D79" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="79" spans="1:4" ht="46.5">
-      <c r="A79" s="4" t="s">
+    <row r="80" spans="1:4" ht="46.5">
+      <c r="A80" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C79" s="4" t="s">
+      <c r="C80" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="D79" s="4" t="s">
+      <c r="D80" s="4" t="s">
         <v>192</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4">
-      <c r="A80" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="C80" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="D80" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="81" spans="1:4">
       <c r="A81" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="4" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="4" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="4" t="s">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="4" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="4" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>128</v>
+        <v>211</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>89</v>
+        <v>211</v>
       </c>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>218</v>
+        <v>128</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>216</v>
+        <v>89</v>
       </c>
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C89" s="4" t="s">
         <v>218</v>
@@ -2413,409 +2435,442 @@
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="4" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>254</v>
+        <v>219</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>255</v>
+        <v>217</v>
       </c>
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>227</v>
+        <v>254</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="4" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="4" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>257</v>
+        <v>231</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>234</v>
+        <v>257</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="4" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>283</v>
+        <v>248</v>
       </c>
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="4" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>249</v>
+        <v>283</v>
       </c>
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>220</v>
+        <v>238</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>282</v>
+        <v>249</v>
       </c>
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>241</v>
+        <v>220</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>252</v>
+        <v>282</v>
       </c>
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="4" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="4" t="s">
-        <v>260</v>
+        <v>244</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>259</v>
+        <v>245</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="4" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="4" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="4" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="4" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="4" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="4" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="4" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="4" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="4" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="4" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="C119" s="6" t="s">
-        <v>308</v>
+        <v>304</v>
+      </c>
+      <c r="C119" s="4" t="s">
+        <v>306</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="C120" s="4" t="s">
-        <v>314</v>
+        <v>307</v>
+      </c>
+      <c r="C120" s="6" t="s">
+        <v>308</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>326</v>
+        <v>309</v>
       </c>
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C121" s="4" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>312</v>
+        <v>326</v>
       </c>
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="4" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="C123" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="D123" s="4" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4">
+      <c r="A124" s="4" t="s">
         <v>320</v>
       </c>
-      <c r="C123" s="4" t="s">
+      <c r="C124" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="D123" s="4" t="s">
+      <c r="D124" s="4" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="124" spans="1:4" ht="139.5">
-      <c r="A124" s="4" t="s">
+    <row r="125" spans="1:4" ht="139.5">
+      <c r="A125" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="C124" s="4" t="s">
+      <c r="C125" s="4" t="s">
         <v>324</v>
       </c>
-      <c r="D124" s="7" t="s">
+      <c r="D125" s="7" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="125" spans="1:4" ht="69.75">
-      <c r="A125" s="4" t="s">
+    <row r="126" spans="1:4" ht="69.75">
+      <c r="A126" s="4" t="s">
         <v>327</v>
       </c>
-      <c r="C125" s="4" t="s">
+      <c r="C126" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="D125" s="4" t="s">
+      <c r="D126" s="4" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="126" spans="1:4">
-      <c r="A126" s="4" t="s">
+    <row r="127" spans="1:4">
+      <c r="A127" s="4" t="s">
         <v>330</v>
       </c>
-      <c r="C126" s="4" t="s">
+      <c r="C127" s="4" t="s">
         <v>332</v>
       </c>
-      <c r="D126" s="4" t="s">
+      <c r="D127" s="4" t="s">
         <v>331</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4">
+      <c r="A128" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="D128" s="4" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4" ht="46.5">
+      <c r="A129" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="C129" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="D129" s="4" t="s">
+        <v>336</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
build(EM): remove CWL dep
</commit_message>
<xml_diff>
--- a/Emmersive/package/LangMod/EN/emmersive_localizations.xlsx
+++ b/Emmersive/package/LangMod/EN/emmersive_localizations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\Elin.Plugins\Emmersive\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84A9C2FE-1A82-4CC9-9A1D-40BA3E8CC610}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD3E26B3-C6A2-4362-9FA3-C32A9115ADBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="28380" windowHeight="17610" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18780" yWindow="1485" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="387" uniqueCount="340">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="343">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1071,10 +1071,19 @@
     <t>em_ui_add_service_deepseek</t>
   </si>
   <si>
-    <t>DeepSeek互換を追加</t>
-  </si>
-  <si>
-    <t>Add DeeSeek</t>
+    <t>Add DeepSeek</t>
+  </si>
+  <si>
+    <t>em_ui_add_service_ollama</t>
+  </si>
+  <si>
+    <t>DeepSeekを追加</t>
+  </si>
+  <si>
+    <t>Ollamaを追加</t>
+  </si>
+  <si>
+    <t>Use Ollama</t>
   </si>
 </sst>
 </file>
@@ -1440,7 +1449,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:XFC129"/>
+  <dimension ref="A1:XFC130"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="23.25"/>
   <cols>
     <col min="1" max="1" width="63.28515625" style="4" customWidth="1"/>
@@ -1584,858 +1593,858 @@
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="4" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="4" t="s">
-        <v>20</v>
+        <v>337</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>142</v>
+        <v>340</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>141</v>
+        <v>338</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C16" s="4" t="s">
         <v>105</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D16" s="4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:4" s="3" customFormat="1">
-      <c r="A16" s="4" t="s">
+    <row r="17" spans="1:4" s="3" customFormat="1">
+      <c r="A17" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4" t="s">
+      <c r="B17" s="4"/>
+      <c r="C17" s="4" t="s">
         <v>106</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D17" s="4" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
+      <c r="A19" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C19" s="4" t="s">
         <v>202</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D19" s="4" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="46.5">
-      <c r="A19" s="4" t="s">
+    <row r="20" spans="1:4" ht="46.5">
+      <c r="A20" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C20" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D20" s="4" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
-      <c r="A20" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="4" t="s">
-        <v>96</v>
+        <v>30</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>97</v>
+        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="4" t="s">
-        <v>222</v>
+        <v>96</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>223</v>
+        <v>109</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>224</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="4" t="s">
-        <v>143</v>
+        <v>222</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>157</v>
+        <v>223</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>153</v>
+        <v>224</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>187</v>
+        <v>167</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>146</v>
+        <v>156</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>152</v>
+        <v>188</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="4" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>189</v>
+        <v>154</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="C33" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
+      <c r="A34" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="C33" s="4" t="s">
+      <c r="C34" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="D33" s="4" t="s">
+      <c r="D34" s="4" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="34" spans="1:4" ht="69.75">
-      <c r="A34" s="4" t="s">
+    <row r="35" spans="1:4" ht="69.75">
+      <c r="A35" s="4" t="s">
         <v>172</v>
       </c>
-      <c r="C34" s="4" t="s">
+      <c r="C35" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="D34" s="4" t="s">
+      <c r="D35" s="4" t="s">
         <v>173</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
-      <c r="A35" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="D35" s="4" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C39" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
+      <c r="A40" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C39" s="4" t="s">
+      <c r="C40" s="4" t="s">
         <v>114</v>
       </c>
-      <c r="D39" s="4" t="s">
+      <c r="D40" s="4" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="40" spans="1:4" s="3" customFormat="1">
-      <c r="A40" s="4" t="s">
+    <row r="41" spans="1:4" s="3" customFormat="1">
+      <c r="A41" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B40" s="4"/>
-      <c r="C40" s="4" t="s">
+      <c r="B41" s="4"/>
+      <c r="C41" s="4" t="s">
         <v>115</v>
       </c>
-      <c r="D40" s="4" t="s">
+      <c r="D41" s="4" t="s">
         <v>76</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4">
-      <c r="A41" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="D41" s="4" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>116</v>
+        <v>136</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>77</v>
+        <v>137</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>117</v>
+        <v>129</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>78</v>
+        <v>90</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4">
+      <c r="A62" s="4" t="s">
         <v>58</v>
       </c>
-      <c r="C61" s="4" t="s">
+      <c r="C62" s="4" t="s">
         <v>122</v>
       </c>
-      <c r="D61" s="4" t="s">
+      <c r="D62" s="4" t="s">
         <v>83</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" s="2" customFormat="1">
-      <c r="A62" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B62" s="4"/>
-      <c r="C62" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="D62" s="4" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="63" spans="1:4" s="2" customFormat="1">
       <c r="A63" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B63" s="4"/>
       <c r="C63" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" s="2" customFormat="1">
+      <c r="A64" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B64" s="4"/>
+      <c r="C64" s="4" t="s">
         <v>124</v>
       </c>
-      <c r="D63" s="4" t="s">
+      <c r="D64" s="4" t="s">
         <v>85</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4">
-      <c r="A64" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C64" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="D64" s="4" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="4" t="s">
-        <v>175</v>
+        <v>70</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>176</v>
+        <v>134</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>176</v>
+        <v>95</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4">
+      <c r="A77" s="4" t="s">
         <v>178</v>
       </c>
-      <c r="C76" s="4" t="s">
+      <c r="C77" s="4" t="s">
         <v>184</v>
       </c>
-      <c r="D76" s="4" t="s">
+      <c r="D77" s="4" t="s">
         <v>184</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" ht="46.5">
-      <c r="A77" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="C77" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="D77" s="4" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="46.5">
       <c r="A78" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" ht="46.5">
+      <c r="A79" s="4" t="s">
         <v>179</v>
       </c>
-      <c r="C78" s="4" t="s">
+      <c r="C79" s="4" t="s">
         <v>185</v>
       </c>
-      <c r="D78" s="4" t="s">
+      <c r="D79" s="4" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="79" spans="1:4">
-      <c r="A79" s="4" t="s">
+    <row r="80" spans="1:4">
+      <c r="A80" s="4" t="s">
         <v>180</v>
       </c>
-      <c r="C79" s="4" t="s">
+      <c r="C80" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="D79" s="4" t="s">
+      <c r="D80" s="4" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="80" spans="1:4" ht="46.5">
-      <c r="A80" s="4" t="s">
+    <row r="81" spans="1:4" ht="46.5">
+      <c r="A81" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="C80" s="4" t="s">
+      <c r="C81" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="D80" s="4" t="s">
+      <c r="D81" s="4" t="s">
         <v>192</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4">
-      <c r="A81" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="C81" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="D81" s="4" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="4" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="4" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="4" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="4" t="s">
-        <v>221</v>
+        <v>205</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="4" t="s">
-        <v>210</v>
+        <v>221</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="4" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>128</v>
+        <v>211</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>89</v>
+        <v>211</v>
       </c>
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>218</v>
+        <v>128</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>216</v>
+        <v>89</v>
       </c>
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C90" s="4" t="s">
         <v>218</v>
@@ -2446,430 +2455,441 @@
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="4" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>254</v>
+        <v>219</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>255</v>
+        <v>217</v>
       </c>
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>227</v>
+        <v>254</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="4" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="4" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>257</v>
+        <v>231</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>234</v>
+        <v>257</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="4" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>283</v>
+        <v>248</v>
       </c>
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="4" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>249</v>
+        <v>283</v>
       </c>
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>220</v>
+        <v>238</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>282</v>
+        <v>249</v>
       </c>
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>241</v>
+        <v>220</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>252</v>
+        <v>282</v>
       </c>
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="4" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="4" t="s">
-        <v>260</v>
+        <v>244</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>259</v>
+        <v>245</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>258</v>
+        <v>250</v>
       </c>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="4" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="4" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="4" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="4" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="4" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="4" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>288</v>
+        <v>281</v>
       </c>
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="4" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="4" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="4" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="4" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="4" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="4" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="4" t="s">
-        <v>307</v>
-      </c>
-      <c r="C120" s="6" t="s">
-        <v>308</v>
+        <v>304</v>
+      </c>
+      <c r="C120" s="4" t="s">
+        <v>306</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="4" t="s">
-        <v>310</v>
-      </c>
-      <c r="C121" s="4" t="s">
-        <v>314</v>
+        <v>307</v>
+      </c>
+      <c r="C121" s="6" t="s">
+        <v>308</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>326</v>
+        <v>309</v>
       </c>
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>312</v>
+        <v>326</v>
       </c>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="4" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="D123" s="4" t="s">
-        <v>319</v>
+        <v>312</v>
       </c>
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="4" t="s">
+        <v>317</v>
+      </c>
+      <c r="C124" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="D124" s="4" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="125" spans="1:4">
+      <c r="A125" s="4" t="s">
         <v>320</v>
       </c>
-      <c r="C124" s="4" t="s">
+      <c r="C125" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="D124" s="4" t="s">
+      <c r="D125" s="4" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="125" spans="1:4" ht="139.5">
-      <c r="A125" s="4" t="s">
+    <row r="126" spans="1:4" ht="139.5">
+      <c r="A126" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="C125" s="4" t="s">
+      <c r="C126" s="4" t="s">
         <v>324</v>
       </c>
-      <c r="D125" s="7" t="s">
+      <c r="D126" s="7" t="s">
         <v>325</v>
       </c>
     </row>
-    <row r="126" spans="1:4" ht="69.75">
-      <c r="A126" s="4" t="s">
+    <row r="127" spans="1:4" ht="69.75">
+      <c r="A127" s="4" t="s">
         <v>327</v>
       </c>
-      <c r="C126" s="4" t="s">
+      <c r="C127" s="4" t="s">
         <v>329</v>
       </c>
-      <c r="D126" s="4" t="s">
+      <c r="D127" s="4" t="s">
         <v>328</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4">
-      <c r="A127" s="4" t="s">
-        <v>330</v>
-      </c>
-      <c r="C127" s="4" t="s">
-        <v>332</v>
-      </c>
-      <c r="D127" s="4" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="C128" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="D128" s="4" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="129" spans="1:4">
+      <c r="A129" s="4" t="s">
         <v>334</v>
       </c>
-      <c r="C128" s="4" t="s">
+      <c r="C129" s="4" t="s">
         <v>333</v>
       </c>
-      <c r="D128" s="4" t="s">
+      <c r="D129" s="4" t="s">
         <v>333</v>
       </c>
     </row>
-    <row r="129" spans="1:4" ht="46.5">
-      <c r="A129" s="4" t="s">
+    <row r="130" spans="1:4" ht="46.5">
+      <c r="A130" s="4" t="s">
         <v>335</v>
       </c>
-      <c r="C129" s="4" t="s">
+      <c r="C130" s="4" t="s">
         <v>336</v>
       </c>
-      <c r="D129" s="4" t="s">
+      <c r="D130" s="4" t="s">
         <v>336</v>
       </c>
     </row>

</xml_diff>

<commit_message>
feat!(EM): character memory module & summarizer
</commit_message>
<xml_diff>
--- a/Emmersive/package/LangMod/EN/emmersive_localizations.xlsx
+++ b/Emmersive/package/LangMod/EN/emmersive_localizations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\Elin.Plugins\Emmersive\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD3E26B3-C6A2-4362-9FA3-C32A9115ADBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C87AED-5457-4413-A136-955EF6F30600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18780" yWindow="1485" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="376">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -62,9 +62,6 @@
     <t>AI Service</t>
   </si>
   <si>
-    <t>Prompt Setting</t>
-  </si>
-  <si>
     <t>Debug Panel</t>
   </si>
   <si>
@@ -328,27 +325,6 @@
   </si>
   <si>
     <t>Reload</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AIサービス  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">プロンプト設定  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">デバッグパネル  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">確認  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">削除  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">テスト生成  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Google Geminiを追加  </t>
   </si>
   <si>
     <t xml:space="preserve">現在のモデル  </t>
@@ -704,9 +680,6 @@
     <t>部屋の中で</t>
   </si>
   <si>
-    <t>キャラクターの絆</t>
-  </si>
-  <si>
     <t>em_character_data_conditions</t>
   </si>
   <si>
@@ -1005,12 +978,6 @@
   </si>
   <si>
     <t>em_ui_chat_keymap</t>
-  </si>
-  <si>
-    <t>チャットボタンをバインド</t>
-  </si>
-  <si>
-    <t>Bind Chat Key</t>
   </si>
   <si>
     <t>em_ui_warn_say_something</t>
@@ -1085,12 +1052,144 @@
   <si>
     <t>Use Ollama</t>
   </si>
+  <si>
+    <t>Prompts</t>
+  </si>
+  <si>
+    <t>Debug</t>
+  </si>
+  <si>
+    <t>Prompt</t>
+  </si>
+  <si>
+    <t>AIサービス</t>
+  </si>
+  <si>
+    <t>確認</t>
+  </si>
+  <si>
+    <t>削除</t>
+  </si>
+  <si>
+    <t>テスト生成</t>
+  </si>
+  <si>
+    <t>Google Geminiを追加</t>
+  </si>
+  <si>
+    <t>絆</t>
+  </si>
+  <si>
+    <t>em_ui_tab_memory</t>
+  </si>
+  <si>
+    <t>Memory</t>
+  </si>
+  <si>
+    <t>em_ui_npc_memory</t>
+  </si>
+  <si>
+    <t>Character Memory</t>
+  </si>
+  <si>
+    <t>em_ui_no_memories</t>
+  </si>
+  <si>
+    <t>Nothing at the moment</t>
+  </si>
+  <si>
+    <t>現在は何もありません</t>
+  </si>
+  <si>
+    <t>Bind Chat Key: {0}</t>
+  </si>
+  <si>
+    <t>チャットボタンをバインド : {0}</t>
+  </si>
+  <si>
+    <t>em_ui_stm_header</t>
+  </si>
+  <si>
+    <t>em_ui_ltm_header</t>
+  </si>
+  <si>
+    <t>em_ui_no_ltm</t>
+  </si>
+  <si>
+    <t>em_ui_summarize_now</t>
+  </si>
+  <si>
+    <t>em_ui_add_ltm</t>
+  </si>
+  <si>
+    <t>em_ui_clear_memory</t>
+  </si>
+  <si>
+    <t>em_ui_edit_memory</t>
+  </si>
+  <si>
+    <t>Edit Character's Memory Data. (Short Memory + Long Memory)</t>
+  </si>
+  <si>
+    <t>Clear All Memory</t>
+  </si>
+  <si>
+    <t>Summarize Now</t>
+  </si>
+  <si>
+    <t>Add New Fact</t>
+  </si>
+  <si>
+    <t>No long time memory yet.</t>
+  </si>
+  <si>
+    <t>まだ長期記憶はありません。</t>
+  </si>
+  <si>
+    <t>要約</t>
+  </si>
+  <si>
+    <t>事実を追加</t>
+  </si>
+  <si>
+    <t>すべての記憶をクリア</t>
+  </si>
+  <si>
+    <t>ャラクターの記憶データを編集（短期記憶＋長期記憶）</t>
+  </si>
+  <si>
+    <t>記憶</t>
+  </si>
+  <si>
+    <t>キャラクター記憶</t>
+  </si>
+  <si>
+    <t>短期記憶（最近の出来事）: {0}</t>
+  </si>
+  <si>
+    <t>長期記憶（事実）: {0}</t>
+  </si>
+  <si>
+    <t>Long Time Memory, Facts : {0}</t>
+  </si>
+  <si>
+    <t>Short Time Memory, Happened Recently : {0}</t>
+  </si>
+  <si>
+    <t>em_ui_summarizing</t>
+  </si>
+  <si>
+    <t>Summarizing…</t>
+  </si>
+  <si>
+    <t>要約中…</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1133,6 +1232,12 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1154,7 +1259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1169,6 +1274,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1449,7 +1555,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:XFC130"/>
+  <dimension ref="A1:XFC141"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="23.25"/>
   <cols>
     <col min="1" max="1" width="63.28515625" style="4" customWidth="1"/>
@@ -1491,16 +1597,16 @@
     </row>
     <row r="4" spans="1:4" s="5" customFormat="1" ht="23.25" customHeight="1">
       <c r="A4" s="4" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -1508,7 +1614,7 @@
         <v>5</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>98</v>
+        <v>335</v>
       </c>
       <c r="D5" s="4" t="s">
         <v>8</v>
@@ -1519,10 +1625,10 @@
         <v>6</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>99</v>
+        <v>334</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>9</v>
+        <v>332</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1530,1367 +1636,1488 @@
         <v>7</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>100</v>
+        <v>333</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>11</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>337</v>
+      </c>
+      <c r="D9" s="4" t="s">
         <v>13</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>338</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>339</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="4" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>342</v>
+        <v>331</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="4" t="s">
-        <v>337</v>
+        <v>326</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>21</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:4" s="3" customFormat="1">
       <c r="A17" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B17" s="4"/>
       <c r="C17" s="4" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>25</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="D18" s="4" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="46.5">
       <c r="A20" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D20" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="D21" s="4" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>96</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="4" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="4" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="4" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="69.75">
       <c r="A35" s="4" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="4" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41" spans="1:4" s="3" customFormat="1">
       <c r="A41" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>137</v>
+        <v>129</v>
       </c>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="51" spans="1:4">
       <c r="A51" s="4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="52" spans="1:4">
       <c r="A52" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="53" spans="1:4">
       <c r="A53" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="54" spans="1:4">
       <c r="A54" s="4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="55" spans="1:4">
       <c r="A55" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C55" s="4" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="D55" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="56" spans="1:4">
       <c r="A56" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="D56" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="57" spans="1:4">
       <c r="A57" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C57" s="4" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="D57" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="58" spans="1:4">
       <c r="A58" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C58" s="4" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="D58" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="59" spans="1:4">
       <c r="A59" s="4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C59" s="4" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="D59" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="60" spans="1:4">
       <c r="A60" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C60" s="4" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="D60" s="4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="61" spans="1:4">
       <c r="A61" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C61" s="4" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="D61" s="4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="62" spans="1:4">
       <c r="A62" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C62" s="4" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="D62" s="4" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="63" spans="1:4" s="2" customFormat="1">
       <c r="A63" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B63" s="4"/>
       <c r="C63" s="4" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D63" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="64" spans="1:4" s="2" customFormat="1">
       <c r="A64" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B64" s="4"/>
       <c r="C64" s="4" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D64" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="65" spans="1:4">
       <c r="A65" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="D65" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="66" spans="1:4">
       <c r="A66" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C66" s="4" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="D66" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="67" spans="1:4">
       <c r="A67" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C67" s="4" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="D67" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="68" spans="1:4">
       <c r="A68" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C68" s="4" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="D68" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="69" spans="1:4">
       <c r="A69" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C69" s="4" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="D69" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="70" spans="1:4">
       <c r="A70" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C70" s="4" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="D70" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="71" spans="1:4">
       <c r="A71" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C71" s="4" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="D71" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="72" spans="1:4">
       <c r="A72" s="4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C72" s="4" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="D72" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="73" spans="1:4">
       <c r="A73" s="4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C73" s="4" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="D73" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="74" spans="1:4">
       <c r="A74" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C74" s="4" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="D74" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="75" spans="1:4">
       <c r="A75" s="4" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
       <c r="C75" s="4" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
       <c r="D75" s="4" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
     </row>
     <row r="76" spans="1:4">
       <c r="A76" s="4" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="C76" s="4" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
       <c r="D76" s="4" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
     </row>
     <row r="77" spans="1:4">
       <c r="A77" s="4" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
       <c r="C77" s="4" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="D77" s="4" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="46.5">
       <c r="A78" s="4" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
       <c r="C78" s="4" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
       <c r="D78" s="4" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
     </row>
     <row r="79" spans="1:4" ht="46.5">
       <c r="A79" s="4" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="C79" s="4" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
       <c r="D79" s="4" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
     </row>
     <row r="80" spans="1:4">
       <c r="A80" s="4" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="C80" s="4" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
       <c r="D80" s="4" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="46.5">
       <c r="A81" s="4" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
       <c r="C81" s="4" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
       <c r="D81" s="4" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
     </row>
     <row r="82" spans="1:4">
       <c r="A82" s="4" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
       <c r="C82" s="4" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
       <c r="D82" s="4" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
     </row>
     <row r="83" spans="1:4">
       <c r="A83" s="4" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="C83" s="4" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="D83" s="4" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="84" spans="1:4">
       <c r="A84" s="4" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="C84" s="4" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
       <c r="D84" s="4" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
     </row>
     <row r="85" spans="1:4">
       <c r="A85" s="4" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="C85" s="4" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="D85" s="4" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
     </row>
     <row r="86" spans="1:4">
       <c r="A86" s="4" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="C86" s="4" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="D86" s="4" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
     </row>
     <row r="87" spans="1:4">
       <c r="A87" s="4" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="C87" s="4" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="D87" s="4" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
     </row>
     <row r="88" spans="1:4">
       <c r="A88" s="4" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="C88" s="4" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="D88" s="4" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
     </row>
     <row r="89" spans="1:4">
       <c r="A89" s="4" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="C89" s="4" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="D89" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="90" spans="1:4">
       <c r="A90" s="4" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
       <c r="C90" s="4" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="D90" s="4" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
     </row>
     <row r="91" spans="1:4">
       <c r="A91" s="4" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="C91" s="4" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="D91" s="4" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
     </row>
     <row r="92" spans="1:4">
       <c r="A92" s="4" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="C92" s="4" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="D92" s="4" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
     </row>
     <row r="93" spans="1:4">
       <c r="A93" s="4" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C93" s="4" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="D93" s="4" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
     </row>
     <row r="94" spans="1:4">
       <c r="A94" s="4" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="C94" s="4" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="D94" s="4" t="s">
-        <v>246</v>
+        <v>237</v>
       </c>
     </row>
     <row r="95" spans="1:4">
       <c r="A95" s="4" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="C95" s="4" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="D95" s="4" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
     </row>
     <row r="96" spans="1:4">
       <c r="A96" s="4" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="C96" s="4" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="D96" s="4" t="s">
-        <v>251</v>
+        <v>242</v>
       </c>
     </row>
     <row r="97" spans="1:4">
       <c r="A97" s="4" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="C97" s="4" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="D97" s="4" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
     </row>
     <row r="98" spans="1:4">
       <c r="A98" s="4" t="s">
-        <v>233</v>
+        <v>224</v>
       </c>
       <c r="C98" s="4" t="s">
-        <v>234</v>
+        <v>225</v>
       </c>
       <c r="D98" s="4" t="s">
-        <v>248</v>
+        <v>239</v>
       </c>
     </row>
     <row r="99" spans="1:4">
       <c r="A99" s="4" t="s">
-        <v>235</v>
+        <v>226</v>
       </c>
       <c r="C99" s="4" t="s">
-        <v>236</v>
+        <v>227</v>
       </c>
       <c r="D99" s="4" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
     </row>
     <row r="100" spans="1:4">
       <c r="A100" s="4" t="s">
-        <v>237</v>
+        <v>228</v>
       </c>
       <c r="C100" s="4" t="s">
-        <v>238</v>
+        <v>229</v>
       </c>
       <c r="D100" s="4" t="s">
-        <v>249</v>
+        <v>240</v>
       </c>
     </row>
     <row r="101" spans="1:4">
       <c r="A101" s="4" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="C101" s="4" t="s">
-        <v>220</v>
+        <v>340</v>
       </c>
       <c r="D101" s="4" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
     </row>
     <row r="102" spans="1:4">
       <c r="A102" s="4" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="C102" s="4" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="D102" s="4" t="s">
-        <v>252</v>
+        <v>243</v>
       </c>
     </row>
     <row r="103" spans="1:4">
       <c r="A103" s="4" t="s">
-        <v>242</v>
+        <v>233</v>
       </c>
       <c r="C103" s="4" t="s">
-        <v>243</v>
+        <v>234</v>
       </c>
       <c r="D103" s="4" t="s">
-        <v>253</v>
+        <v>244</v>
       </c>
     </row>
     <row r="104" spans="1:4">
       <c r="A104" s="4" t="s">
-        <v>244</v>
+        <v>235</v>
       </c>
       <c r="C104" s="4" t="s">
-        <v>245</v>
+        <v>236</v>
       </c>
       <c r="D104" s="4" t="s">
-        <v>250</v>
+        <v>241</v>
       </c>
     </row>
     <row r="105" spans="1:4">
       <c r="A105" s="4" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="C105" s="4" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="D105" s="4" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
     </row>
     <row r="106" spans="1:4">
       <c r="A106" s="4" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="C106" s="4" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="D106" s="4" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
     </row>
     <row r="107" spans="1:4">
       <c r="A107" s="4" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="C107" s="4" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
     </row>
     <row r="108" spans="1:4">
       <c r="A108" s="4" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="C108" s="4" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
     </row>
     <row r="109" spans="1:4">
       <c r="A109" s="4" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="C109" s="4" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
     </row>
     <row r="110" spans="1:4">
       <c r="A110" s="4" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="C110" s="4" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
     </row>
     <row r="111" spans="1:4">
       <c r="A111" s="4" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="C111" s="4" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
     </row>
     <row r="112" spans="1:4">
       <c r="A112" s="4" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="C112" s="4" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="D112" s="4" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
     </row>
     <row r="113" spans="1:4">
       <c r="A113" s="4" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
       <c r="C113" s="4" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
     </row>
     <row r="114" spans="1:4">
       <c r="A114" s="4" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="C114" s="4" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
     </row>
     <row r="115" spans="1:4">
       <c r="A115" s="4" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="C115" s="4" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="D115" s="4" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
     </row>
     <row r="116" spans="1:4">
       <c r="A116" s="4" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="C116" s="4" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>293</v>
+        <v>284</v>
       </c>
     </row>
     <row r="117" spans="1:4">
       <c r="A117" s="4" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="C117" s="4" t="s">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
     </row>
     <row r="118" spans="1:4">
       <c r="A118" s="4" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="C118" s="4" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="D118" s="4" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
     </row>
     <row r="119" spans="1:4">
       <c r="A119" s="4" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="C119" s="4" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="D119" s="4" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
     </row>
     <row r="120" spans="1:4">
       <c r="A120" s="4" t="s">
-        <v>304</v>
+        <v>295</v>
       </c>
       <c r="C120" s="4" t="s">
-        <v>306</v>
+        <v>297</v>
       </c>
       <c r="D120" s="4" t="s">
-        <v>305</v>
+        <v>296</v>
       </c>
     </row>
     <row r="121" spans="1:4">
       <c r="A121" s="4" t="s">
-        <v>307</v>
+        <v>298</v>
       </c>
       <c r="C121" s="6" t="s">
-        <v>308</v>
+        <v>299</v>
       </c>
       <c r="D121" s="4" t="s">
-        <v>309</v>
+        <v>300</v>
       </c>
     </row>
     <row r="122" spans="1:4">
       <c r="A122" s="4" t="s">
-        <v>310</v>
+        <v>301</v>
       </c>
       <c r="C122" s="4" t="s">
-        <v>314</v>
+        <v>305</v>
       </c>
       <c r="D122" s="4" t="s">
-        <v>326</v>
+        <v>315</v>
       </c>
     </row>
     <row r="123" spans="1:4">
       <c r="A123" s="4" t="s">
-        <v>311</v>
+        <v>302</v>
       </c>
       <c r="C123" s="4" t="s">
-        <v>313</v>
+        <v>304</v>
       </c>
       <c r="D123" s="4" t="s">
-        <v>312</v>
+        <v>303</v>
       </c>
     </row>
     <row r="124" spans="1:4">
       <c r="A124" s="4" t="s">
-        <v>317</v>
+        <v>308</v>
       </c>
       <c r="C124" s="4" t="s">
-        <v>318</v>
+        <v>309</v>
       </c>
       <c r="D124" s="4" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
     </row>
     <row r="125" spans="1:4">
       <c r="A125" s="4" t="s">
-        <v>320</v>
+        <v>311</v>
       </c>
       <c r="C125" s="4" t="s">
-        <v>321</v>
+        <v>349</v>
       </c>
       <c r="D125" s="4" t="s">
-        <v>322</v>
+        <v>348</v>
       </c>
     </row>
     <row r="126" spans="1:4" ht="139.5">
       <c r="A126" s="4" t="s">
-        <v>323</v>
+        <v>312</v>
       </c>
       <c r="C126" s="4" t="s">
-        <v>324</v>
+        <v>313</v>
       </c>
       <c r="D126" s="7" t="s">
-        <v>325</v>
+        <v>314</v>
       </c>
     </row>
     <row r="127" spans="1:4" ht="69.75">
       <c r="A127" s="4" t="s">
-        <v>327</v>
+        <v>316</v>
       </c>
       <c r="C127" s="4" t="s">
-        <v>329</v>
+        <v>318</v>
       </c>
       <c r="D127" s="4" t="s">
-        <v>328</v>
+        <v>317</v>
       </c>
     </row>
     <row r="128" spans="1:4">
       <c r="A128" s="4" t="s">
-        <v>330</v>
+        <v>319</v>
       </c>
       <c r="C128" s="4" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
       <c r="D128" s="4" t="s">
-        <v>331</v>
+        <v>320</v>
       </c>
     </row>
     <row r="129" spans="1:4">
       <c r="A129" s="4" t="s">
-        <v>334</v>
+        <v>323</v>
       </c>
       <c r="C129" s="4" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="D129" s="4" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
     </row>
     <row r="130" spans="1:4" ht="46.5">
       <c r="A130" s="4" t="s">
-        <v>335</v>
+        <v>324</v>
       </c>
       <c r="C130" s="4" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="D130" s="4" t="s">
-        <v>336</v>
+        <v>325</v>
+      </c>
+    </row>
+    <row r="131" spans="1:4">
+      <c r="A131" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="C131" s="8" t="s">
+        <v>367</v>
+      </c>
+      <c r="D131" s="4" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="132" spans="1:4">
+      <c r="A132" s="4" t="s">
+        <v>343</v>
+      </c>
+      <c r="C132" s="8" t="s">
+        <v>368</v>
+      </c>
+      <c r="D132" s="4" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="133" spans="1:4">
+      <c r="A133" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="C133" s="8" t="s">
+        <v>347</v>
+      </c>
+      <c r="D133" s="4" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="134" spans="1:4">
+      <c r="A134" s="4" t="s">
+        <v>350</v>
+      </c>
+      <c r="C134" s="4" t="s">
+        <v>369</v>
+      </c>
+      <c r="D134" s="4" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="135" spans="1:4">
+      <c r="A135" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="C135" s="4" t="s">
+        <v>370</v>
+      </c>
+      <c r="D135" s="4" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="136" spans="1:4">
+      <c r="A136" s="4" t="s">
+        <v>352</v>
+      </c>
+      <c r="C136" s="4" t="s">
+        <v>362</v>
+      </c>
+      <c r="D136" s="4" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="137" spans="1:4">
+      <c r="A137" s="4" t="s">
+        <v>353</v>
+      </c>
+      <c r="C137" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="D137" s="4" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="138" spans="1:4">
+      <c r="A138" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="C138" s="4" t="s">
+        <v>364</v>
+      </c>
+      <c r="D138" s="4" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="139" spans="1:4">
+      <c r="A139" s="4" t="s">
+        <v>355</v>
+      </c>
+      <c r="C139" s="4" t="s">
+        <v>365</v>
+      </c>
+      <c r="D139" s="4" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="140" spans="1:4">
+      <c r="A140" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="C140" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="D140" s="4" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="141" spans="1:4">
+      <c r="A141" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="C141" s="4" t="s">
+        <v>375</v>
+      </c>
+      <c r="D141" s="4" t="s">
+        <v>374</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(EM): improved configurable memory settings
</commit_message>
<xml_diff>
--- a/Emmersive/package/LangMod/EN/emmersive_localizations.xlsx
+++ b/Emmersive/package/LangMod/EN/emmersive_localizations.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\Elin.Plugins\Emmersive\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49C87AED-5457-4413-A136-955EF6F30600}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59C3148D-D85C-4DAA-AF6E-F38EBB90A69E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18780" yWindow="1485" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="382">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1183,6 +1183,24 @@
   </si>
   <si>
     <t>要約中…</t>
+  </si>
+  <si>
+    <t>em_ui_memory_prompt</t>
+  </si>
+  <si>
+    <t>Summarizer Prompt</t>
+  </si>
+  <si>
+    <t>サマライザープロンプト</t>
+  </si>
+  <si>
+    <t>em_ui_summarize_done</t>
+  </si>
+  <si>
+    <t>Summarized</t>
+  </si>
+  <si>
+    <t>要約ok</t>
   </si>
 </sst>
 </file>
@@ -1555,7 +1573,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:XFC141"/>
+  <dimension ref="A1:XFC143"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="23.25"/>
   <cols>
     <col min="1" max="1" width="63.28515625" style="4" customWidth="1"/>
@@ -3120,6 +3138,28 @@
         <v>374</v>
       </c>
     </row>
+    <row r="142" spans="1:4">
+      <c r="A142" s="4" t="s">
+        <v>376</v>
+      </c>
+      <c r="C142" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="D142" s="4" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="143" spans="1:4">
+      <c r="A143" s="4" t="s">
+        <v>379</v>
+      </c>
+      <c r="C143" s="4" t="s">
+        <v>381</v>
+      </c>
+      <c r="D143" s="4" t="s">
+        <v>380</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat(EM): disable summarization by default
</commit_message>
<xml_diff>
--- a/Emmersive/package/LangMod/EN/emmersive_localizations.xlsx
+++ b/Emmersive/package/LangMod/EN/emmersive_localizations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\Elin.Plugins\Emmersive\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59C3148D-D85C-4DAA-AF6E-F38EBB90A69E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72EECEEA-8420-48FC-9A1F-19CCC4DEE64A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18780" yWindow="1485" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8340" yWindow="2685" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="385">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1201,6 +1201,15 @@
   </si>
   <si>
     <t>要約ok</t>
+  </si>
+  <si>
+    <t>em_ui_use_summarize</t>
+  </si>
+  <si>
+    <t>Enable Memory Summarization</t>
+  </si>
+  <si>
+    <t>記憶の要約をオン</t>
   </si>
 </sst>
 </file>
@@ -1573,7 +1582,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:XFC143"/>
+  <dimension ref="A1:XFC144"/>
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="23.25"/>
   <cols>
     <col min="1" max="1" width="63.28515625" style="4" customWidth="1"/>
@@ -3160,6 +3169,17 @@
         <v>380</v>
       </c>
     </row>
+    <row r="144" spans="1:4">
+      <c r="A144" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="C144" s="4" t="s">
+        <v>384</v>
+      </c>
+      <c r="D144" s="4" t="s">
+        <v>383</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>